<commit_message>
cambios en la data
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\github\seguimiento_cdd_fest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F7D2BB-05EB-4B89-AB5E-C8AC86F0571E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2734D496-9B18-4116-8D14-79BF67534BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="92">
   <si>
     <t>1054-2026</t>
   </si>
@@ -225,6 +225,9 @@
     <t>Requiere reprogramación</t>
   </si>
   <si>
+    <t>Preliminar (en reuniones y revisión previa)</t>
+  </si>
+  <si>
     <t>mma_estado</t>
   </si>
   <si>
@@ -289,9 +292,6 @@
   </si>
   <si>
     <t>Dificultades para la adquisición de equipos, los mismos que están en levantamiento de observaciones de las EETT.</t>
-  </si>
-  <si>
-    <t>Si Aprobado</t>
   </si>
   <si>
     <t>Difucltades para conseguir material de hilo y profesionales técnicos</t>
@@ -311,6 +311,12 @@
   </si>
   <si>
     <t>--</t>
+  </si>
+  <si>
+    <t>Aprobado (elaboración de informe a emitir)</t>
+  </si>
+  <si>
+    <t>Demora en adquisición de equipo heperbarico, debido a los tiempos de contratación de mayor cuantía, así como su fabricación, importación y desaduanaje.</t>
   </si>
 </sst>
 </file>
@@ -321,11 +327,18 @@
     <numFmt numFmtId="8" formatCode="&quot;S/&quot;\ #,##0.00;[Red]\-&quot;S/&quot;\ #,##0.00"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -401,9 +414,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -412,23 +425,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -708,28 +725,28 @@
         <v>46</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="10" t="s">
-        <v>76</v>
+      <c r="K1" s="16" t="s">
+        <v>77</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>48</v>
       </c>
       <c r="N1" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="P1" s="1" t="s">
         <v>49</v>
@@ -738,10 +755,10 @@
         <v>50</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -796,8 +813,11 @@
       <c r="Q2" t="s">
         <v>38</v>
       </c>
-      <c r="R2" s="3" t="s">
-        <v>39</v>
+      <c r="R2" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -846,11 +866,11 @@
       <c r="Q3" t="s">
         <v>38</v>
       </c>
-      <c r="R3" s="3" t="s">
-        <v>83</v>
+      <c r="R3" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -899,8 +919,8 @@
       <c r="Q4" t="s">
         <v>38</v>
       </c>
-      <c r="R4" s="3" t="s">
-        <v>83</v>
+      <c r="R4" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S4" s="5" t="s">
         <v>84</v>
@@ -952,8 +972,8 @@
       <c r="Q5" t="s">
         <v>38</v>
       </c>
-      <c r="R5" s="3" t="s">
-        <v>39</v>
+      <c r="R5" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S5" s="5" t="s">
         <v>85</v>
@@ -1011,8 +1031,8 @@
       <c r="Q6" t="s">
         <v>38</v>
       </c>
-      <c r="R6" s="3" t="s">
-        <v>39</v>
+      <c r="R6" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S6" s="15" t="s">
         <v>86</v>
@@ -1070,8 +1090,8 @@
       <c r="Q7" t="s">
         <v>38</v>
       </c>
-      <c r="R7" s="3" t="s">
-        <v>39</v>
+      <c r="R7" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S7" s="5" t="s">
         <v>87</v>
@@ -1123,11 +1143,11 @@
       <c r="Q8" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="3" t="s">
-        <v>39</v>
+      <c r="R8" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S8" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1176,11 +1196,11 @@
       <c r="Q9" t="s">
         <v>38</v>
       </c>
-      <c r="R9" s="3" t="s">
+      <c r="R9" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="S9" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="S9" s="5" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1230,7 +1250,7 @@
         <v>38</v>
       </c>
       <c r="R10" s="3" t="s">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="S10" s="5" t="s">
         <v>88</v>
@@ -1288,11 +1308,8 @@
       <c r="Q11" t="s">
         <v>39</v>
       </c>
-      <c r="R11" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="S11" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1347,11 +1364,8 @@
       <c r="Q12" t="s">
         <v>39</v>
       </c>
-      <c r="R12" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="S12" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1406,11 +1420,8 @@
       <c r="Q13" t="s">
         <v>39</v>
       </c>
-      <c r="R13" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="S13" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1459,9 +1470,6 @@
       <c r="Q14" t="s">
         <v>39</v>
       </c>
-      <c r="R14" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="S14" s="5" t="s">
         <v>89</v>
       </c>
@@ -1518,9 +1526,6 @@
       <c r="Q15" t="s">
         <v>39</v>
       </c>
-      <c r="R15" s="3" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="16" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16">
@@ -1568,11 +1573,11 @@
       <c r="Q16" t="s">
         <v>38</v>
       </c>
-      <c r="R16" s="3" t="s">
-        <v>39</v>
+      <c r="R16" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S16" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1627,11 +1632,11 @@
       <c r="Q17" t="s">
         <v>38</v>
       </c>
-      <c r="R17" s="3" t="s">
-        <v>39</v>
+      <c r="R17" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S17" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1686,11 +1691,11 @@
       <c r="Q18" t="s">
         <v>38</v>
       </c>
-      <c r="R18" s="3" t="s">
-        <v>39</v>
+      <c r="R18" s="17" t="s">
+        <v>90</v>
       </c>
       <c r="S18" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1739,11 +1744,8 @@
       <c r="Q19" t="s">
         <v>39</v>
       </c>
-      <c r="R19" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="S19" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1826,10 +1828,10 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -1842,10 +1844,10 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -1866,18 +1868,18 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualización de nombre de variable
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\github\seguimiento_cdd_fest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2734D496-9B18-4116-8D14-79BF67534BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF80B58-5028-4B80-97B3-5BF114AB0B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejecutivo" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="93">
   <si>
     <t>1054-2026</t>
   </si>
@@ -317,6 +317,9 @@
   </si>
   <si>
     <t>Demora en adquisición de equipo heperbarico, debido a los tiempos de contratación de mayor cuantía, así como su fabricación, importación y desaduanaje.</t>
+  </si>
+  <si>
+    <t>Incidencias reportadas</t>
   </si>
 </sst>
 </file>
@@ -327,11 +330,18 @@
     <numFmt numFmtId="8" formatCode="&quot;S/&quot;\ #,##0.00;[Red]\-&quot;S/&quot;\ #,##0.00"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -414,9 +424,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -425,28 +435,29 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1878,8 +1889,8 @@
       <c r="A15" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>69</v>
+      <c r="B15" s="18" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualización de datos 5 columnas
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\github\seguimiento_cdd_fest\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF80B58-5028-4B80-97B3-5BF114AB0B0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C4F4A03-5012-4B68-B77A-2B455B6B795E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejecutivo" sheetId="1" r:id="rId1"/>
@@ -288,12 +288,6 @@
     <t>N ha logrado la contratación de los 3 TDR, Seguimiento, analista y eléctrico; ademáss 1 servicio de abril. A ese personal, el cual su contrato sale en agosto.</t>
   </si>
   <si>
-    <t>Cite postergó inicio de actividades</t>
-  </si>
-  <si>
-    <t>Dificultades para la adquisición de equipos, los mismos que están en levantamiento de observaciones de las EETT.</t>
-  </si>
-  <si>
     <t>Difucltades para conseguir material de hilo y profesionales técnicos</t>
   </si>
   <si>
@@ -307,9 +301,6 @@
     <t>Servicios de terceros programadas para el mes 1 por retrasos se programaron al mes 2 de ejecución actividades 1.2 y 1.4.</t>
   </si>
   <si>
-    <t>De las 8 actividades programadas para el hito 1, 6 de ellas corresponden al RSM3. Con respecto a las otras 02 actividades (actividad 2.1 y 2.6), la UT menciona que se va a reportar para el hito 1 como "en proceso" ya que no se va culminar de ejecutar porque actualmente se encuentra en proceso el nuevo requerimiento, dado la situación la UT solicitará modificación de menor alcance.</t>
-  </si>
-  <si>
     <t>--</t>
   </si>
   <si>
@@ -320,15 +311,26 @@
   </si>
   <si>
     <t>Incidencias reportadas</t>
+  </si>
+  <si>
+    <t>Dificultades para la adquisición de equipos/insumos para de ensayos de laboratorio, los mismos que están en levantamiento de observaciones de las EETT.</t>
+  </si>
+  <si>
+    <t>La UT Lima tiene 06 actividades para el Hito 1, 02 actividades se modificaron debido a que se cambió la denominación de las consultorías para que no ingresen al PDP</t>
+  </si>
+  <si>
+    <t>De lo antes señalado, se evidencia que, el sustento de modificación del cronograma del proyecto se sustenta principalmente, a factores asociados a condiciones de clima
+con presencia de lluvias en la región Loreto y disponibilidad de Unidades Productivas para la prestación de los servicios programados en el proyecto.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="8" formatCode="&quot;S/&quot;\ #,##0.00;[Red]\-&quot;S/&quot;\ #,##0.00"/>
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="170" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -424,7 +426,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -446,7 +448,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
@@ -458,10 +459,11 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -744,7 +746,7 @@
       <c r="J1" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="K1" s="16" t="s">
+      <c r="K1" s="15" t="s">
         <v>77</v>
       </c>
       <c r="L1" s="7" t="s">
@@ -788,10 +790,10 @@
       <c r="E2">
         <v>3</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="18">
         <v>2</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2" s="12">
         <v>0.66700000000000004</v>
       </c>
       <c r="H2" s="9">
@@ -800,35 +802,35 @@
       <c r="I2" s="9">
         <v>13</v>
       </c>
-      <c r="J2" s="14">
+      <c r="J2" s="13">
         <v>230221</v>
       </c>
-      <c r="K2" s="14">
+      <c r="K2" s="13">
         <v>230125</v>
       </c>
-      <c r="L2" s="14">
+      <c r="L2" s="13">
         <v>10750</v>
       </c>
-      <c r="M2" s="14">
+      <c r="M2" s="13">
         <v>8238</v>
       </c>
-      <c r="N2" s="12">
+      <c r="N2" s="11">
         <v>1</v>
       </c>
-      <c r="O2" s="12">
+      <c r="O2" s="11">
         <v>4.7E-2</v>
       </c>
-      <c r="P2" s="12">
+      <c r="P2" s="11">
         <v>3.5999999999999997E-2</v>
       </c>
       <c r="Q2" t="s">
         <v>38</v>
       </c>
-      <c r="R2" s="17" t="s">
-        <v>90</v>
+      <c r="R2" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S2" s="5" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -847,38 +849,38 @@
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="18">
         <v>0</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3" s="12">
         <v>0</v>
       </c>
-      <c r="J3" s="14">
+      <c r="J3" s="13">
         <v>223105</v>
       </c>
-      <c r="K3" s="14">
+      <c r="K3" s="13">
         <v>26758</v>
       </c>
-      <c r="L3" s="14">
+      <c r="L3" s="13">
         <v>21778</v>
       </c>
-      <c r="M3" s="14">
+      <c r="M3" s="13">
         <v>1400</v>
       </c>
-      <c r="N3" s="12">
+      <c r="N3" s="11">
         <v>0.12</v>
       </c>
-      <c r="O3" s="12">
+      <c r="O3" s="11">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="P3" s="12">
+      <c r="P3" s="11">
         <v>6.0000000000000001E-3</v>
       </c>
       <c r="Q3" t="s">
         <v>38</v>
       </c>
-      <c r="R3" s="17" t="s">
-        <v>90</v>
+      <c r="R3" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S3" s="5" t="s">
         <v>80</v>
@@ -900,41 +902,41 @@
       <c r="E4">
         <v>13</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="18">
         <v>6</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="12">
         <v>0.46200000000000002</v>
       </c>
-      <c r="J4" s="14">
+      <c r="J4" s="13">
         <v>217442</v>
       </c>
-      <c r="K4" s="14">
+      <c r="K4" s="13">
         <v>87580</v>
       </c>
-      <c r="L4" s="14">
+      <c r="L4" s="13">
         <v>87580</v>
       </c>
-      <c r="M4" s="14">
+      <c r="M4" s="13">
         <v>0</v>
       </c>
-      <c r="N4" s="12">
+      <c r="N4" s="11">
         <v>0.40300000000000002</v>
       </c>
-      <c r="O4" s="12">
+      <c r="O4" s="11">
         <v>0.40300000000000002</v>
       </c>
-      <c r="P4" s="12">
+      <c r="P4" s="11">
         <v>0</v>
       </c>
       <c r="Q4" t="s">
         <v>38</v>
       </c>
-      <c r="R4" s="17" t="s">
-        <v>90</v>
+      <c r="R4" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -953,41 +955,41 @@
       <c r="E5">
         <v>2</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="18">
         <v>0</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="12">
         <v>0</v>
       </c>
-      <c r="J5" s="14">
+      <c r="J5" s="13">
         <v>159704</v>
       </c>
-      <c r="K5" s="14">
+      <c r="K5" s="13">
         <v>116743</v>
       </c>
-      <c r="L5" s="14">
+      <c r="L5" s="13">
         <v>116743</v>
       </c>
-      <c r="M5" s="14">
+      <c r="M5" s="13">
         <v>24898</v>
       </c>
-      <c r="N5" s="12">
+      <c r="N5" s="11">
         <v>0.73099999999999998</v>
       </c>
-      <c r="O5" s="12">
+      <c r="O5" s="11">
         <v>0.73099999999999998</v>
       </c>
-      <c r="P5" s="12">
+      <c r="P5" s="11">
         <v>0.156</v>
       </c>
       <c r="Q5" t="s">
         <v>38</v>
       </c>
-      <c r="R5" s="17" t="s">
-        <v>90</v>
+      <c r="R5" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1006,10 +1008,10 @@
       <c r="E6">
         <v>14</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="18">
         <v>12</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="12">
         <v>0.85699999999999998</v>
       </c>
       <c r="H6" s="9">
@@ -1018,35 +1020,35 @@
       <c r="I6" s="9">
         <v>105</v>
       </c>
-      <c r="J6" s="14">
+      <c r="J6" s="13">
         <v>158350</v>
       </c>
-      <c r="K6" s="14">
+      <c r="K6" s="13">
         <v>79392</v>
       </c>
-      <c r="L6" s="14">
+      <c r="L6" s="13">
         <v>79392</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="13">
         <v>11802</v>
       </c>
-      <c r="N6" s="12">
+      <c r="N6" s="11">
         <v>0.501</v>
       </c>
-      <c r="O6" s="12">
+      <c r="O6" s="11">
         <v>0.501</v>
       </c>
-      <c r="P6" s="12">
+      <c r="P6" s="11">
         <v>7.4999999999999997E-2</v>
       </c>
       <c r="Q6" t="s">
         <v>38</v>
       </c>
-      <c r="R6" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="S6" s="15" t="s">
-        <v>86</v>
+      <c r="R6" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="S6" s="14" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1065,47 +1067,47 @@
       <c r="E7">
         <v>7</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="18">
         <v>6</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="12">
         <v>0.85699999999999998</v>
       </c>
       <c r="H7" s="9">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I7" s="9">
-        <v>16</v>
-      </c>
-      <c r="J7" s="14">
+        <v>20</v>
+      </c>
+      <c r="J7" s="13">
         <v>156838</v>
       </c>
-      <c r="K7" s="14">
+      <c r="K7" s="13">
         <v>112636</v>
       </c>
-      <c r="L7" s="14">
+      <c r="L7" s="13">
         <v>112636</v>
       </c>
-      <c r="M7" s="14">
+      <c r="M7" s="13">
         <v>21968</v>
       </c>
-      <c r="N7" s="12">
+      <c r="N7" s="11">
         <v>0.71799999999999997</v>
       </c>
-      <c r="O7" s="12">
+      <c r="O7" s="11">
         <v>0.71799999999999997</v>
       </c>
-      <c r="P7" s="12">
+      <c r="P7" s="11">
         <v>0.14000000000000001</v>
       </c>
       <c r="Q7" t="s">
         <v>38</v>
       </c>
-      <c r="R7" s="17" t="s">
-        <v>90</v>
+      <c r="R7" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1124,38 +1126,38 @@
       <c r="E8">
         <v>3</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="18">
         <v>0</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="12">
         <v>0</v>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="13">
         <v>147913</v>
       </c>
-      <c r="K8" s="14">
+      <c r="K8" s="13">
         <v>21617</v>
       </c>
-      <c r="L8" s="14">
+      <c r="L8" s="13">
         <v>21611</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="13">
         <v>12494</v>
       </c>
-      <c r="N8" s="12">
+      <c r="N8" s="11">
         <v>0.14599999999999999</v>
       </c>
-      <c r="O8" s="12">
+      <c r="O8" s="11">
         <v>0.14599999999999999</v>
       </c>
-      <c r="P8" s="12">
+      <c r="P8" s="11">
         <v>8.4000000000000005E-2</v>
       </c>
       <c r="Q8" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="17" t="s">
-        <v>90</v>
+      <c r="R8" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S8" s="5" t="s">
         <v>79</v>
@@ -1177,41 +1179,41 @@
       <c r="E9">
         <v>5</v>
       </c>
-      <c r="F9">
-        <v>5</v>
-      </c>
-      <c r="G9" s="13">
+      <c r="F9" s="18">
+        <v>4</v>
+      </c>
+      <c r="G9" s="12">
         <v>1</v>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="13">
         <v>109375</v>
       </c>
-      <c r="K9" s="14">
+      <c r="K9" s="13">
         <v>45000</v>
       </c>
-      <c r="L9" s="14">
+      <c r="L9" s="13">
         <v>45000</v>
       </c>
-      <c r="M9" s="14">
+      <c r="M9" s="13">
         <v>0</v>
       </c>
-      <c r="N9" s="12">
+      <c r="N9" s="11">
         <v>0.41099999999999998</v>
       </c>
-      <c r="O9" s="12">
+      <c r="O9" s="11">
         <v>0.41099999999999998</v>
       </c>
-      <c r="P9" s="12">
+      <c r="P9" s="11">
         <v>0</v>
       </c>
       <c r="Q9" t="s">
         <v>38</v>
       </c>
-      <c r="R9" s="17" t="s">
+      <c r="R9" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="S9" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="S9" s="5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1230,31 +1232,31 @@
       <c r="E10">
         <v>8</v>
       </c>
-      <c r="F10" s="11">
-        <v>8</v>
-      </c>
-      <c r="G10" s="13">
+      <c r="F10" s="18">
+        <v>6</v>
+      </c>
+      <c r="G10" s="12">
         <v>1</v>
       </c>
-      <c r="J10" s="14">
+      <c r="J10" s="13">
         <v>103175</v>
       </c>
-      <c r="K10" s="14">
+      <c r="K10" s="13">
         <v>52874</v>
       </c>
-      <c r="L10" s="14">
+      <c r="L10" s="13">
         <v>52874</v>
       </c>
-      <c r="M10" s="14">
+      <c r="M10" s="13">
         <v>38594</v>
       </c>
-      <c r="N10" s="12">
+      <c r="N10" s="11">
         <v>0.51200000000000001</v>
       </c>
-      <c r="O10" s="12">
+      <c r="O10" s="11">
         <v>0.51200000000000001</v>
       </c>
-      <c r="P10" s="12">
+      <c r="P10" s="11">
         <v>0.374</v>
       </c>
       <c r="Q10" t="s">
@@ -1264,7 +1266,7 @@
         <v>61</v>
       </c>
       <c r="S10" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1283,10 +1285,10 @@
       <c r="E11">
         <v>4</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="18">
         <v>4</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="12">
         <v>1</v>
       </c>
       <c r="H11" s="9">
@@ -1295,25 +1297,25 @@
       <c r="I11" s="9">
         <v>7</v>
       </c>
-      <c r="J11" s="14">
+      <c r="J11" s="13">
         <v>96950</v>
       </c>
-      <c r="K11" s="14">
+      <c r="K11" s="13">
         <v>96355</v>
       </c>
-      <c r="L11" s="14">
+      <c r="L11" s="13">
         <v>96355</v>
       </c>
-      <c r="M11" s="14">
+      <c r="M11" s="13">
         <v>23736</v>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="11">
         <v>0.99399999999999999</v>
       </c>
-      <c r="O11" s="12">
+      <c r="O11" s="11">
         <v>0.99399999999999999</v>
       </c>
-      <c r="P11" s="12">
+      <c r="P11" s="11">
         <v>0.245</v>
       </c>
       <c r="Q11" t="s">
@@ -1339,37 +1341,37 @@
       <c r="E12">
         <v>3</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="18">
         <v>3</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="12">
         <v>1</v>
       </c>
       <c r="H12" s="9">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I12" s="9">
-        <v>66</v>
-      </c>
-      <c r="J12" s="14">
+        <v>67</v>
+      </c>
+      <c r="J12" s="13">
         <v>96875</v>
       </c>
-      <c r="K12" s="14">
+      <c r="K12" s="13">
         <v>85400</v>
       </c>
-      <c r="L12" s="14">
+      <c r="L12" s="13">
         <v>85400</v>
       </c>
-      <c r="M12" s="14">
+      <c r="M12" s="13">
         <v>59000</v>
       </c>
-      <c r="N12" s="12">
+      <c r="N12" s="11">
         <v>0.88200000000000001</v>
       </c>
-      <c r="O12" s="12">
+      <c r="O12" s="11">
         <v>0.88200000000000001</v>
       </c>
-      <c r="P12" s="12">
+      <c r="P12" s="11">
         <v>0.60899999999999999</v>
       </c>
       <c r="Q12" t="s">
@@ -1395,37 +1397,37 @@
       <c r="E13">
         <v>12</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="18">
         <v>12</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="12">
         <v>1</v>
       </c>
       <c r="H13" s="9">
-        <v>165</v>
+        <v>115</v>
       </c>
       <c r="I13" s="9">
         <v>74</v>
       </c>
-      <c r="J13" s="14">
+      <c r="J13" s="13">
         <v>95775</v>
       </c>
-      <c r="K13" s="14">
+      <c r="K13" s="13">
         <v>87700</v>
       </c>
-      <c r="L13" s="14">
+      <c r="L13" s="13">
         <v>87700</v>
       </c>
-      <c r="M13" s="14">
+      <c r="M13" s="13">
         <v>25900</v>
       </c>
-      <c r="N13" s="12">
+      <c r="N13" s="11">
         <v>0.91600000000000004</v>
       </c>
-      <c r="O13" s="12">
+      <c r="O13" s="11">
         <v>0.91600000000000004</v>
       </c>
-      <c r="P13" s="12">
+      <c r="P13" s="11">
         <v>0.27</v>
       </c>
       <c r="Q13" t="s">
@@ -1451,38 +1453,38 @@
       <c r="E14">
         <v>5</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="18">
         <v>5</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="12">
         <v>1</v>
       </c>
-      <c r="J14" s="14">
+      <c r="J14" s="13">
         <v>89665</v>
       </c>
-      <c r="K14" s="14">
+      <c r="K14" s="13">
         <v>65474</v>
       </c>
-      <c r="L14" s="14">
+      <c r="L14" s="13">
         <v>60075</v>
       </c>
-      <c r="M14" s="14">
+      <c r="M14" s="13">
         <v>8910</v>
       </c>
-      <c r="N14" s="12">
+      <c r="N14" s="11">
         <v>0.73</v>
       </c>
-      <c r="O14" s="12">
+      <c r="O14" s="11">
         <v>0.67</v>
       </c>
-      <c r="P14" s="12">
+      <c r="P14" s="11">
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="Q14" t="s">
         <v>39</v>
       </c>
       <c r="S14" s="5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1501,10 +1503,10 @@
       <c r="E15">
         <v>8</v>
       </c>
-      <c r="F15">
-        <v>6</v>
-      </c>
-      <c r="G15" s="13">
+      <c r="F15" s="18">
+        <v>8</v>
+      </c>
+      <c r="G15" s="12">
         <v>0.75</v>
       </c>
       <c r="H15" s="9">
@@ -1513,25 +1515,25 @@
       <c r="I15" s="9">
         <v>22</v>
       </c>
-      <c r="J15" s="14">
+      <c r="J15" s="13">
         <v>78375</v>
       </c>
-      <c r="K15" s="14">
+      <c r="K15" s="13">
         <v>67950</v>
       </c>
-      <c r="L15" s="14">
+      <c r="L15" s="13">
         <v>67950</v>
       </c>
-      <c r="M15" s="14">
+      <c r="M15" s="13">
         <v>41300</v>
       </c>
-      <c r="N15" s="12">
+      <c r="N15" s="11">
         <v>0.86699999999999999</v>
       </c>
-      <c r="O15" s="12">
+      <c r="O15" s="11">
         <v>0.86699999999999999</v>
       </c>
-      <c r="P15" s="12">
+      <c r="P15" s="11">
         <v>0.52700000000000002</v>
       </c>
       <c r="Q15" t="s">
@@ -1554,38 +1556,38 @@
       <c r="E16">
         <v>4</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="18">
         <v>2</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="12">
         <v>0.5</v>
       </c>
-      <c r="J16" s="14">
+      <c r="J16" s="13">
         <v>70675</v>
       </c>
-      <c r="K16" s="14">
+      <c r="K16" s="13">
         <v>64403</v>
       </c>
-      <c r="L16" s="14">
+      <c r="L16" s="13">
         <v>64403</v>
       </c>
-      <c r="M16" s="14">
+      <c r="M16" s="13">
         <v>0</v>
       </c>
-      <c r="N16" s="12">
+      <c r="N16" s="11">
         <v>0.91100000000000003</v>
       </c>
-      <c r="O16" s="12">
+      <c r="O16" s="11">
         <v>0.91100000000000003</v>
       </c>
-      <c r="P16" s="12">
+      <c r="P16" s="11">
         <v>0</v>
       </c>
       <c r="Q16" t="s">
         <v>38</v>
       </c>
-      <c r="R16" s="17" t="s">
-        <v>90</v>
+      <c r="R16" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S16" s="5" t="s">
         <v>67</v>
@@ -1607,10 +1609,10 @@
       <c r="E17">
         <v>13</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="18">
         <v>7</v>
       </c>
-      <c r="G17" s="13">
+      <c r="G17" s="12">
         <v>0.53800000000000003</v>
       </c>
       <c r="H17" s="9">
@@ -1619,35 +1621,35 @@
       <c r="I17" s="9">
         <v>5</v>
       </c>
-      <c r="J17" s="14">
+      <c r="J17" s="13">
         <v>56175</v>
       </c>
-      <c r="K17" s="14">
+      <c r="K17" s="13">
         <v>45000</v>
       </c>
-      <c r="L17" s="14">
+      <c r="L17" s="13">
         <v>45000</v>
       </c>
-      <c r="M17" s="14">
+      <c r="M17" s="13">
         <v>0</v>
       </c>
-      <c r="N17" s="12">
+      <c r="N17" s="11">
         <v>0.80100000000000005</v>
       </c>
-      <c r="O17" s="12">
+      <c r="O17" s="11">
         <v>0.80100000000000005</v>
       </c>
-      <c r="P17" s="12">
+      <c r="P17" s="11">
         <v>0</v>
       </c>
       <c r="Q17" t="s">
         <v>38</v>
       </c>
-      <c r="R17" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="S17" s="5" t="s">
-        <v>82</v>
+      <c r="R17" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="S17" s="14" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1666,44 +1668,44 @@
       <c r="E18">
         <v>8</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="18">
         <v>5</v>
       </c>
-      <c r="G18" s="13">
+      <c r="G18" s="12">
         <v>0.625</v>
       </c>
       <c r="H18" s="9">
+        <v>7</v>
+      </c>
+      <c r="I18" s="9">
         <v>6</v>
       </c>
-      <c r="I18" s="9">
-        <v>5</v>
-      </c>
-      <c r="J18" s="14">
+      <c r="J18" s="13">
         <v>40975</v>
       </c>
-      <c r="K18" s="14">
+      <c r="K18" s="13">
         <v>26000</v>
       </c>
-      <c r="L18" s="14">
+      <c r="L18" s="13">
         <v>26000</v>
       </c>
-      <c r="M18" s="14">
+      <c r="M18" s="13">
         <v>5500</v>
       </c>
-      <c r="N18" s="12">
+      <c r="N18" s="11">
         <v>0.63500000000000001</v>
       </c>
-      <c r="O18" s="12">
+      <c r="O18" s="11">
         <v>0.63500000000000001</v>
       </c>
-      <c r="P18" s="12">
+      <c r="P18" s="11">
         <v>0.13400000000000001</v>
       </c>
       <c r="Q18" t="s">
         <v>38</v>
       </c>
-      <c r="R18" s="17" t="s">
-        <v>90</v>
+      <c r="R18" s="16" t="s">
+        <v>87</v>
       </c>
       <c r="S18" s="5" t="s">
         <v>81</v>
@@ -1725,31 +1727,31 @@
       <c r="E19">
         <v>2</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="18">
         <v>2</v>
       </c>
-      <c r="G19" s="13">
+      <c r="G19" s="12">
         <v>1</v>
       </c>
-      <c r="J19" s="14">
+      <c r="J19" s="13">
         <v>19131</v>
       </c>
-      <c r="K19" s="14">
+      <c r="K19" s="13">
         <v>12925</v>
       </c>
-      <c r="L19" s="14">
+      <c r="L19" s="13">
         <v>12925</v>
       </c>
-      <c r="M19" s="14">
+      <c r="M19" s="13">
         <v>2000</v>
       </c>
-      <c r="N19" s="12">
+      <c r="N19" s="11">
         <v>0.67600000000000005</v>
       </c>
-      <c r="O19" s="12">
+      <c r="O19" s="11">
         <v>0.67600000000000005</v>
       </c>
-      <c r="P19" s="12">
+      <c r="P19" s="11">
         <v>0.105</v>
       </c>
       <c r="Q19" t="s">
@@ -1889,8 +1891,8 @@
       <c r="A15" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>92</v>
+      <c r="B15" s="17" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>